<commit_message>
Merged production code to feature/intranet branch
</commit_message>
<xml_diff>
--- a/Portland_Gas_DB_Design.xlsx
+++ b/Portland_Gas_DB_Design.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Index" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Identity" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Identity" sheetId="2" state="hidden" r:id="rId2"/>
     <sheet name="Documents" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Approval" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="All Requests" sheetId="5" state="visible" r:id="rId5"/>
@@ -16,7 +16,7 @@
     <sheet name="Assets" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Intranet" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="Notifications" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Future Extras" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Future Extras" sheetId="10" state="hidden" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -797,7 +797,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F41"/>
+  <dimension ref="A1:F39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -817,7 +817,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Schema Reference  ·  v7.0  ·  June 2026</t>
+          <t>Schema Reference  ·  v8.0  ·  June 2026</t>
         </is>
       </c>
     </row>
@@ -858,81 +858,81 @@
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Identity &amp; Organisation</t>
+          <t>Document Library</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Identity</t>
+          <t>Documents</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>documents</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>~200</t>
+          <t>thousands</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Authentication records only — one row per login account</t>
+          <t>Unified file &amp; folder store — self-referencing parent_id for unlimited nesting. type='folder' has no file_path.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>Identity &amp; Organisation</t>
+          <t>Approval Workflow Engine</t>
         </is>
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>Identity</t>
+          <t>Approval</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>employees</t>
+          <t>approval_workflows</t>
         </is>
       </c>
       <c r="D8" s="10" t="inlineStr">
         <is>
-          <t>~200</t>
+          <t>hundreds</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>Business/HR identity — bridges to users; all workflow FKs point here</t>
+          <t>Named workflow templates — one per process type</t>
         </is>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Document Library</t>
+          <t>Approval Workflow Engine</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Documents</t>
+          <t>Approval</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>documents</t>
+          <t>workflow_steps</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>thousands</t>
+          <t>hundreds</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Unified file &amp; folder store — self-referencing parent_id for unlimited nesting. type='folder' has no file_path.</t>
+          <t>Ordered steps within a workflow template. assignee_type drives how the approver is resolved at runtime.</t>
         </is>
       </c>
     </row>
@@ -949,7 +949,7 @@
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>approval_workflows</t>
+          <t>approval_requests</t>
         </is>
       </c>
       <c r="D10" s="10" t="inlineStr">
@@ -959,7 +959,7 @@
       </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>Named workflow templates — one per process type</t>
+          <t>Live tracker — one row per request entering a workflow. current_step_number advances on each approval.</t>
         </is>
       </c>
     </row>
@@ -976,17 +976,17 @@
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>workflow_steps</t>
+          <t>approval_step_assignments</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>hundreds</t>
+          <t>thousands</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Ordered steps within a workflow template. assignee_type drives how the approver is resolved at runtime.</t>
+          <t>Stores the resolved approver for each step of each request. Created when a step becomes active.</t>
         </is>
       </c>
     </row>
@@ -1003,17 +1003,17 @@
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>approval_requests</t>
+          <t>approval_history</t>
         </is>
       </c>
       <c r="D12" s="10" t="inlineStr">
         <is>
-          <t>hundreds</t>
+          <t>thousands</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>Live tracker — one row per request entering a workflow. current_step_number advances on each approval.</t>
+          <t>Immutable step-by-step log of approver actions — one row per approval action. Never updated, only inserted.</t>
         </is>
       </c>
     </row>
@@ -1030,7 +1030,7 @@
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>approval_step_assignments</t>
+          <t>workflow_audit_trail</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
@@ -1040,7 +1040,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>Stores the resolved approver for each step of each request. Created when a step becomes active — either resolved from the workflow template or captured from the requester's people-picker selection.</t>
+          <t>Standalone audit trail written by workflowEngine.audit(). Captures every actor event across all workflow requests — both requester actions (submitted, recalled, returned) and approver actions (approved, rejected, escalated). Called independently from the engine so any service can write to it.</t>
         </is>
       </c>
     </row>
@@ -1057,17 +1057,17 @@
       </c>
       <c r="C14" s="9" t="inlineStr">
         <is>
-          <t>approval_history</t>
+          <t>approver_groups</t>
         </is>
       </c>
       <c r="D14" s="10" t="inlineStr">
         <is>
-          <t>thousands</t>
+          <t>hundreds</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr">
         <is>
-          <t>Immutable audit log — one row per action taken. Never updated, only inserted.</t>
+          <t>Named lists of people for requester_pick steps — not role-based, manually curated by admin</t>
         </is>
       </c>
     </row>
@@ -1084,7 +1084,7 @@
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>approver_groups</t>
+          <t>approver_group_members</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
@@ -1094,7 +1094,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>Named lists of people for requester_pick steps — not role-based, manually curated by admin</t>
+          <t>Members belonging to an approver group — many employees can belong to many groups</t>
         </is>
       </c>
     </row>
@@ -1111,7 +1111,7 @@
       </c>
       <c r="C16" s="9" t="inlineStr">
         <is>
-          <t>approver_group_members</t>
+          <t>workflow_assignments</t>
         </is>
       </c>
       <c r="D16" s="10" t="inlineStr">
@@ -1121,24 +1121,24 @@
       </c>
       <c r="E16" s="8" t="inlineStr">
         <is>
-          <t>Members belonging to an approver group — many employees can belong to many groups</t>
+          <t>Maps each process/request_type to its active workflow — tells the engine which workflow to trigger</t>
         </is>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>Approval Workflow Engine</t>
+          <t>All Requests</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Approval</t>
+          <t>All Requests</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>workflow_assignments</t>
+          <t>all_requests</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
@@ -1148,24 +1148,24 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>Maps each process/request_type to its active workflow — tells the engine which workflow to trigger</t>
+          <t>Unified registry of every request across all processes — powers the All Requests dashboard. Updated on each status change.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>All Requests</t>
+          <t>Procurement</t>
         </is>
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>All Requests</t>
+          <t>Procurement</t>
         </is>
       </c>
       <c r="C18" s="9" t="inlineStr">
         <is>
-          <t>all_requests</t>
+          <t>vendors</t>
         </is>
       </c>
       <c r="D18" s="10" t="inlineStr">
@@ -1175,7 +1175,7 @@
       </c>
       <c r="E18" s="8" t="inlineStr">
         <is>
-          <t>Unified registry of every request across all processes — powers the All Requests dashboard view</t>
+          <t>Unified vendor registry — permanent (approved company suppliers) and temporary (ad-hoc one-time vendors entered at request time). Filter by vendor_type to separate them. procurement_request_id is null for permanent vendors.</t>
         </is>
       </c>
     </row>
@@ -1192,7 +1192,7 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>vendors</t>
+          <t>procurement_requests</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
@@ -1202,7 +1202,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>Approved supplier/vendor registry</t>
+          <t>Purchase/procurement request raised by any employee</t>
         </is>
       </c>
     </row>
@@ -1219,7 +1219,7 @@
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>one_time_vendors</t>
+          <t>procurement_items</t>
         </is>
       </c>
       <c r="D20" s="10" t="inlineStr">
@@ -1229,7 +1229,7 @@
       </c>
       <c r="E20" s="8" t="inlineStr">
         <is>
-          <t>Temporary/ad-hoc vendors entered at request time — not part of the approved vendor registry</t>
+          <t>Line items on a procurement request</t>
         </is>
       </c>
     </row>
@@ -1246,7 +1246,7 @@
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>procurement_requests</t>
+          <t>purchase_orders</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
@@ -1256,24 +1256,24 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>Purchase/procurement request raised by any employee</t>
+          <t>PO issued after procurement request is fully approved</t>
         </is>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="8" t="inlineStr">
         <is>
-          <t>Procurement</t>
+          <t>Asset Management</t>
         </is>
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t>Procurement</t>
+          <t>Assets</t>
         </is>
       </c>
       <c r="C22" s="9" t="inlineStr">
         <is>
-          <t>procurement_items</t>
+          <t>asset_categories</t>
         </is>
       </c>
       <c r="D22" s="10" t="inlineStr">
@@ -1283,24 +1283,24 @@
       </c>
       <c r="E22" s="8" t="inlineStr">
         <is>
-          <t>Line items on a procurement request</t>
+          <t>Asset type classification</t>
         </is>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>Procurement</t>
+          <t>Asset Management</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>Procurement</t>
+          <t>Assets</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>purchase_orders</t>
+          <t>assets</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
@@ -1310,7 +1310,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>PO issued after procurement request is fully approved</t>
+          <t>Individual asset register</t>
         </is>
       </c>
     </row>
@@ -1327,7 +1327,7 @@
       </c>
       <c r="C24" s="9" t="inlineStr">
         <is>
-          <t>asset_categories</t>
+          <t>asset_requests</t>
         </is>
       </c>
       <c r="D24" s="10" t="inlineStr">
@@ -1337,7 +1337,7 @@
       </c>
       <c r="E24" s="8" t="inlineStr">
         <is>
-          <t>Asset type classification</t>
+          <t>Employee request to purchase, borrow, or repair an asset</t>
         </is>
       </c>
     </row>
@@ -1354,7 +1354,7 @@
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>assets</t>
+          <t>asset_assignment_logs</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
@@ -1364,7 +1364,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>Individual asset register</t>
+          <t>Tracks who an asset was assigned to and when it was returned</t>
         </is>
       </c>
     </row>
@@ -1381,7 +1381,7 @@
       </c>
       <c r="C26" s="9" t="inlineStr">
         <is>
-          <t>asset_requests</t>
+          <t>asset_maintenance_logs</t>
         </is>
       </c>
       <c r="D26" s="10" t="inlineStr">
@@ -1391,24 +1391,24 @@
       </c>
       <c r="E26" s="8" t="inlineStr">
         <is>
-          <t>Employee request to purchase, borrow, or repair an asset</t>
+          <t>Maintenance and repair history per asset</t>
         </is>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>Asset Management</t>
+          <t>Intranet Content</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>Assets</t>
+          <t>Intranet</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>asset_assignment_logs</t>
+          <t>intranet_announcements</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
@@ -1418,24 +1418,24 @@
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>Tracks who an asset was assigned to and when it was returned</t>
+          <t>News and announcements published on the intranet</t>
         </is>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="8" t="inlineStr">
         <is>
-          <t>Asset Management</t>
+          <t>Intranet Content</t>
         </is>
       </c>
       <c r="B28" s="8" t="inlineStr">
         <is>
-          <t>Assets</t>
+          <t>Intranet</t>
         </is>
       </c>
       <c r="C28" s="9" t="inlineStr">
         <is>
-          <t>asset_maintenance_logs</t>
+          <t>intranet_events</t>
         </is>
       </c>
       <c r="D28" s="10" t="inlineStr">
@@ -1445,7 +1445,7 @@
       </c>
       <c r="E28" s="8" t="inlineStr">
         <is>
-          <t>Maintenance and repair history per asset</t>
+          <t>Company events listed on the intranet events page</t>
         </is>
       </c>
     </row>
@@ -1462,7 +1462,7 @@
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>intranet_announcements</t>
+          <t>intranet_spotlight</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr">
@@ -1472,7 +1472,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>News and announcements published on the intranet</t>
+          <t>Employee spotlight and recognition — covers employee of the month, long service, achievements</t>
         </is>
       </c>
     </row>
@@ -1489,7 +1489,7 @@
       </c>
       <c r="C30" s="9" t="inlineStr">
         <is>
-          <t>intranet_events</t>
+          <t>intranet_message_from</t>
         </is>
       </c>
       <c r="D30" s="10" t="inlineStr">
@@ -1499,7 +1499,7 @@
       </c>
       <c r="E30" s="8" t="inlineStr">
         <is>
-          <t>Company events listed on the intranet events page</t>
+          <t>Message from MD or leadership — typically one active record at a time</t>
         </is>
       </c>
     </row>
@@ -1516,7 +1516,7 @@
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>intranet_spotlight</t>
+          <t>intranet_quick_links</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
@@ -1526,7 +1526,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>Employee spotlight and recognition — covers employee of the month, long service, achievements</t>
+          <t>Quick-access links shown on the intranet home page</t>
         </is>
       </c>
     </row>
@@ -1543,7 +1543,7 @@
       </c>
       <c r="C32" s="9" t="inlineStr">
         <is>
-          <t>intranet_message_from</t>
+          <t>intranet_feedback</t>
         </is>
       </c>
       <c r="D32" s="10" t="inlineStr">
@@ -1553,7 +1553,7 @@
       </c>
       <c r="E32" s="8" t="inlineStr">
         <is>
-          <t>Message from MD or leadership — typically one active record at a time</t>
+          <t>Staff feedback and suggestions submitted via the intranet</t>
         </is>
       </c>
     </row>
@@ -1570,7 +1570,7 @@
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>intranet_quick_links</t>
+          <t>intranet_faq</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr">
@@ -1580,151 +1580,97 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>Quick-access links shown on the intranet home page</t>
+          <t>FAQ entries managed via admin portal</t>
         </is>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="8" t="inlineStr">
         <is>
-          <t>Intranet Content</t>
+          <t>Notifications</t>
         </is>
       </c>
       <c r="B34" s="8" t="inlineStr">
         <is>
-          <t>Intranet</t>
+          <t>Notifications</t>
         </is>
       </c>
       <c r="C34" s="9" t="inlineStr">
         <is>
-          <t>intranet_feedback</t>
+          <t>notifications</t>
         </is>
       </c>
       <c r="D34" s="10" t="inlineStr">
         <is>
-          <t>hundreds</t>
+          <t>thousands</t>
         </is>
       </c>
       <c r="E34" s="8" t="inlineStr">
         <is>
-          <t>Staff feedback and suggestions submitted via the intranet</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="18" customHeight="1">
-      <c r="A35" s="5" t="inlineStr">
-        <is>
-          <t>Intranet Content</t>
-        </is>
-      </c>
-      <c r="B35" s="5" t="inlineStr">
-        <is>
-          <t>Intranet</t>
-        </is>
-      </c>
-      <c r="C35" s="6" t="inlineStr">
-        <is>
-          <t>intranet_faq</t>
-        </is>
-      </c>
-      <c r="D35" s="7" t="inlineStr">
-        <is>
-          <t>hundreds</t>
-        </is>
-      </c>
-      <c r="E35" s="5" t="inlineStr">
-        <is>
-          <t>FAQ entries managed via admin portal</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="8" t="inlineStr">
-        <is>
-          <t>Notifications</t>
-        </is>
-      </c>
-      <c r="B36" s="8" t="inlineStr">
-        <is>
-          <t>Notifications</t>
-        </is>
-      </c>
-      <c r="C36" s="9" t="inlineStr">
-        <is>
-          <t>notifications</t>
-        </is>
-      </c>
-      <c r="D36" s="10" t="inlineStr">
-        <is>
-          <t>thousands</t>
-        </is>
-      </c>
-      <c r="E36" s="8" t="inlineStr">
-        <is>
           <t>In-app notifications sent to employees — also used to trigger emails</t>
         </is>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" s="11" t="inlineStr">
+        <is>
+          <t>Legend</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  PK</t>
+        </is>
+      </c>
+      <c r="B37" s="13" t="inlineStr">
+        <is>
+          <t>Primary Key</t>
+        </is>
+      </c>
+      <c r="C37" s="14" t="n"/>
+      <c r="D37" s="14" t="n"/>
+      <c r="E37" s="15" t="n"/>
+    </row>
     <row r="38">
-      <c r="A38" s="11" t="inlineStr">
-        <is>
-          <t>Legend</t>
-        </is>
-      </c>
+      <c r="A38" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  FK</t>
+        </is>
+      </c>
+      <c r="B38" s="13" t="inlineStr">
+        <is>
+          <t>Foreign Key — references another table</t>
+        </is>
+      </c>
+      <c r="C38" s="14" t="n"/>
+      <c r="D38" s="14" t="n"/>
+      <c r="E38" s="15" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  PK</t>
+      <c r="A39" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  NULL</t>
         </is>
       </c>
       <c r="B39" s="13" t="inlineStr">
         <is>
-          <t>Primary Key</t>
+          <t>Column is nullable (YES in Nullable column)</t>
         </is>
       </c>
       <c r="C39" s="14" t="n"/>
       <c r="D39" s="14" t="n"/>
       <c r="E39" s="15" t="n"/>
     </row>
-    <row r="40">
-      <c r="A40" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  FK</t>
-        </is>
-      </c>
-      <c r="B40" s="13" t="inlineStr">
-        <is>
-          <t>Foreign Key — references another table</t>
-        </is>
-      </c>
-      <c r="C40" s="14" t="n"/>
-      <c r="D40" s="14" t="n"/>
-      <c r="E40" s="15" t="n"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  NULL</t>
-        </is>
-      </c>
-      <c r="B41" s="13" t="inlineStr">
-        <is>
-          <t>Column is nullable (YES in Nullable column)</t>
-        </is>
-      </c>
-      <c r="C41" s="14" t="n"/>
-      <c r="D41" s="14" t="n"/>
-      <c r="E41" s="15" t="n"/>
-    </row>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="B40:E40"/>
-    <mergeCell ref="B41:E41"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="B38:E38"/>
     <mergeCell ref="B39:E39"/>
     <mergeCell ref="A4:F4"/>
+    <mergeCell ref="B37:E37"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2932,7 +2878,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G97"/>
+  <dimension ref="A1:G112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -3678,7 +3624,7 @@
     <row r="47" ht="30" customHeight="1">
       <c r="A47" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Stores the resolved approver for each step of each request. Created when a step becomes active — either resolved from the workflow template or captured from the requester's people-picker selection.</t>
+          <t xml:space="preserve">  Stores the resolved approver for each step of each request. Created when a step becomes active.</t>
         </is>
       </c>
     </row>
@@ -3820,7 +3766,7 @@
     <row r="57" ht="30" customHeight="1">
       <c r="A57" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Immutable audit log — one row per action taken. Never updated, only inserted.</t>
+          <t xml:space="preserve">  Immutable step-by-step log of approver actions — one row per approval action. Never updated, only inserted.</t>
         </is>
       </c>
     </row>
@@ -3999,14 +3945,14 @@
     <row r="68" ht="24" customHeight="1">
       <c r="A68" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">  approver_groups</t>
+          <t xml:space="preserve">  workflow_audit_trail</t>
         </is>
       </c>
     </row>
     <row r="69" ht="30" customHeight="1">
       <c r="A69" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Named lists of people for requester_pick steps — not role-based, manually curated by admin</t>
+          <t xml:space="preserve">  Standalone audit trail written by workflowEngine.audit(). Captures every actor event across all workflow requests — both requester actions (submitted, recalled, returned) and approver actions (approved, rejected, escalated). Called independently from the engine so any service can write to it.</t>
         </is>
       </c>
     </row>
@@ -4055,54 +4001,58 @@
       </c>
     </row>
     <row r="72" ht="17" customHeight="1">
-      <c r="A72" s="26" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="B72" s="26" t="inlineStr">
-        <is>
-          <t>VARCHAR(100)</t>
-        </is>
-      </c>
-      <c r="C72" s="27" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D72" s="28" t="inlineStr">
-        <is>
-          <t>e.g. SODA Approvers, Executive Committee</t>
+      <c r="A72" s="32" t="inlineStr">
+        <is>
+          <t>workflow_id</t>
+        </is>
+      </c>
+      <c r="B72" s="33" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="C72" s="34" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D72" s="35" t="inlineStr">
+        <is>
+          <t>FK → approval_workflows.id</t>
         </is>
       </c>
     </row>
     <row r="73" ht="17" customHeight="1">
-      <c r="A73" s="5" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="B73" s="5" t="inlineStr">
-        <is>
-          <t>TEXT</t>
-        </is>
-      </c>
-      <c r="C73" s="31" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="D73" s="30" t="inlineStr"/>
+      <c r="A73" s="22" t="inlineStr">
+        <is>
+          <t>request_id</t>
+        </is>
+      </c>
+      <c r="B73" s="23" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="C73" s="24" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D73" s="25" t="inlineStr">
+        <is>
+          <t>PK of the originating request row</t>
+        </is>
+      </c>
     </row>
     <row r="74" ht="17" customHeight="1">
       <c r="A74" s="26" t="inlineStr">
         <is>
-          <t>is_active</t>
+          <t>request_type</t>
         </is>
       </c>
       <c r="B74" s="26" t="inlineStr">
         <is>
-          <t>BOOLEAN</t>
+          <t>VARCHAR(50)</t>
         </is>
       </c>
       <c r="C74" s="27" t="inlineStr">
@@ -4112,14 +4062,14 @@
       </c>
       <c r="D74" s="28" t="inlineStr">
         <is>
-          <t>default true</t>
+          <t>procurement | asset</t>
         </is>
       </c>
     </row>
     <row r="75" ht="17" customHeight="1">
       <c r="A75" s="32" t="inlineStr">
         <is>
-          <t>created_by</t>
+          <t>actor_id</t>
         </is>
       </c>
       <c r="B75" s="33" t="inlineStr">
@@ -4134,364 +4084,618 @@
       </c>
       <c r="D75" s="35" t="inlineStr">
         <is>
-          <t>FK → employees.id</t>
+          <t>FK → employees.id — person who performed the action</t>
         </is>
       </c>
     </row>
     <row r="76" ht="17" customHeight="1">
       <c r="A76" s="26" t="inlineStr">
         <is>
-          <t>created_at</t>
+          <t>actor_role</t>
         </is>
       </c>
       <c r="B76" s="26" t="inlineStr">
         <is>
-          <t>TIMESTAMPTZ</t>
-        </is>
-      </c>
-      <c r="C76" s="27" t="inlineStr">
-        <is>
-          <t>NO</t>
+          <t>VARCHAR(80)</t>
+        </is>
+      </c>
+      <c r="C76" s="38" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
       <c r="D76" s="28" t="inlineStr">
         <is>
-          <t>default now()</t>
+          <t>role in this request e.g. requester | line_manager | hod | finance_manager | md</t>
         </is>
       </c>
     </row>
     <row r="77" ht="17" customHeight="1">
       <c r="A77" s="5" t="inlineStr">
         <is>
+          <t>step_number</t>
+        </is>
+      </c>
+      <c r="B77" s="5" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="C77" s="31" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D77" s="30" t="inlineStr">
+        <is>
+          <t>null for requester-initiated actions (submitted, recalled)</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="17" customHeight="1">
+      <c r="A78" s="26" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
+      <c r="B78" s="26" t="inlineStr">
+        <is>
+          <t>VARCHAR(40)</t>
+        </is>
+      </c>
+      <c r="C78" s="27" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D78" s="28" t="inlineStr">
+        <is>
+          <t>submitted | approved | rejected | returned | escalated | recalled</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="17" customHeight="1">
+      <c r="A79" s="5" t="inlineStr">
+        <is>
+          <t>comment</t>
+        </is>
+      </c>
+      <c r="B79" s="5" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="C79" s="31" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D79" s="30" t="inlineStr">
+        <is>
+          <t>approver note or requester comment</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="17" customHeight="1">
+      <c r="A80" s="26" t="inlineStr">
+        <is>
+          <t>acted_at</t>
+        </is>
+      </c>
+      <c r="B80" s="26" t="inlineStr">
+        <is>
+          <t>TIMESTAMPTZ</t>
+        </is>
+      </c>
+      <c r="C80" s="27" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D80" s="28" t="inlineStr">
+        <is>
+          <t>default now()</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="24" customHeight="1">
+      <c r="A83" s="39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  approver_groups</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="30" customHeight="1">
+      <c r="A84" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Named lists of people for requester_pick steps — not role-based, manually curated by admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="18" customHeight="1">
+      <c r="A85" s="21" t="inlineStr">
+        <is>
+          <t>Column</t>
+        </is>
+      </c>
+      <c r="B85" s="21" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C85" s="21" t="inlineStr">
+        <is>
+          <t>Nullable</t>
+        </is>
+      </c>
+      <c r="D85" s="21" t="inlineStr">
+        <is>
+          <t>Notes / FK</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="17" customHeight="1">
+      <c r="A86" s="22" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B86" s="23" t="inlineStr">
+        <is>
+          <t>SERIAL</t>
+        </is>
+      </c>
+      <c r="C86" s="24" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D86" s="25" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="17" customHeight="1">
+      <c r="A87" s="26" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B87" s="26" t="inlineStr">
+        <is>
+          <t>VARCHAR(100)</t>
+        </is>
+      </c>
+      <c r="C87" s="27" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D87" s="28" t="inlineStr">
+        <is>
+          <t>e.g. SODA Approvers, Executive Committee</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="17" customHeight="1">
+      <c r="A88" s="5" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="B88" s="5" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="C88" s="31" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D88" s="30" t="inlineStr"/>
+    </row>
+    <row r="89" ht="17" customHeight="1">
+      <c r="A89" s="26" t="inlineStr">
+        <is>
+          <t>is_active</t>
+        </is>
+      </c>
+      <c r="B89" s="26" t="inlineStr">
+        <is>
+          <t>BOOLEAN</t>
+        </is>
+      </c>
+      <c r="C89" s="27" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D89" s="28" t="inlineStr">
+        <is>
+          <t>default true</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="17" customHeight="1">
+      <c r="A90" s="32" t="inlineStr">
+        <is>
+          <t>created_by</t>
+        </is>
+      </c>
+      <c r="B90" s="33" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="C90" s="34" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D90" s="35" t="inlineStr">
+        <is>
+          <t>FK → employees.id</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="17" customHeight="1">
+      <c r="A91" s="26" t="inlineStr">
+        <is>
+          <t>created_at</t>
+        </is>
+      </c>
+      <c r="B91" s="26" t="inlineStr">
+        <is>
+          <t>TIMESTAMPTZ</t>
+        </is>
+      </c>
+      <c r="C91" s="27" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D91" s="28" t="inlineStr">
+        <is>
+          <t>default now()</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="17" customHeight="1">
+      <c r="A92" s="5" t="inlineStr">
+        <is>
           <t>updated_at</t>
         </is>
       </c>
-      <c r="B77" s="5" t="inlineStr">
+      <c r="B92" s="5" t="inlineStr">
         <is>
           <t>TIMESTAMPTZ</t>
         </is>
       </c>
-      <c r="C77" s="29" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D77" s="30" t="inlineStr">
+      <c r="C92" s="29" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D92" s="30" t="inlineStr">
         <is>
           <t>default now()</t>
         </is>
       </c>
     </row>
-    <row r="80" ht="24" customHeight="1">
-      <c r="A80" s="39" t="inlineStr">
+    <row r="95" ht="24" customHeight="1">
+      <c r="A95" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">  approver_group_members</t>
         </is>
       </c>
     </row>
-    <row r="81" ht="30" customHeight="1">
-      <c r="A81" s="20" t="inlineStr">
+    <row r="96" ht="30" customHeight="1">
+      <c r="A96" s="20" t="inlineStr">
         <is>
           <t xml:space="preserve">  Members belonging to an approver group — many employees can belong to many groups</t>
         </is>
       </c>
     </row>
-    <row r="82" ht="18" customHeight="1">
-      <c r="A82" s="21" t="inlineStr">
+    <row r="97" ht="18" customHeight="1">
+      <c r="A97" s="21" t="inlineStr">
         <is>
           <t>Column</t>
         </is>
       </c>
-      <c r="B82" s="21" t="inlineStr">
+      <c r="B97" s="21" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="C82" s="21" t="inlineStr">
+      <c r="C97" s="21" t="inlineStr">
         <is>
           <t>Nullable</t>
         </is>
       </c>
-      <c r="D82" s="21" t="inlineStr">
+      <c r="D97" s="21" t="inlineStr">
         <is>
           <t>Notes / FK</t>
         </is>
       </c>
     </row>
-    <row r="83" ht="17" customHeight="1">
-      <c r="A83" s="22" t="inlineStr">
+    <row r="98" ht="17" customHeight="1">
+      <c r="A98" s="22" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B83" s="23" t="inlineStr">
+      <c r="B98" s="23" t="inlineStr">
         <is>
           <t>SERIAL</t>
         </is>
       </c>
-      <c r="C83" s="24" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D83" s="25" t="inlineStr">
+      <c r="C98" s="24" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D98" s="25" t="inlineStr">
         <is>
           <t>PK</t>
         </is>
       </c>
     </row>
-    <row r="84" ht="17" customHeight="1">
-      <c r="A84" s="32" t="inlineStr">
+    <row r="99" ht="17" customHeight="1">
+      <c r="A99" s="32" t="inlineStr">
         <is>
           <t>group_id</t>
         </is>
       </c>
-      <c r="B84" s="33" t="inlineStr">
+      <c r="B99" s="33" t="inlineStr">
         <is>
           <t>INT</t>
         </is>
       </c>
-      <c r="C84" s="34" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D84" s="35" t="inlineStr">
+      <c r="C99" s="34" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D99" s="35" t="inlineStr">
         <is>
           <t>FK → approver_groups.id</t>
         </is>
       </c>
     </row>
-    <row r="85" ht="17" customHeight="1">
-      <c r="A85" s="32" t="inlineStr">
+    <row r="100" ht="17" customHeight="1">
+      <c r="A100" s="32" t="inlineStr">
         <is>
           <t>employee_id</t>
         </is>
       </c>
-      <c r="B85" s="33" t="inlineStr">
+      <c r="B100" s="33" t="inlineStr">
         <is>
           <t>INT</t>
         </is>
       </c>
-      <c r="C85" s="34" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D85" s="35" t="inlineStr">
+      <c r="C100" s="34" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D100" s="35" t="inlineStr">
         <is>
           <t>FK → employees.id</t>
         </is>
       </c>
     </row>
-    <row r="86" ht="17" customHeight="1">
-      <c r="A86" s="26" t="inlineStr">
+    <row r="101" ht="17" customHeight="1">
+      <c r="A101" s="26" t="inlineStr">
         <is>
           <t>added_at</t>
         </is>
       </c>
-      <c r="B86" s="26" t="inlineStr">
+      <c r="B101" s="26" t="inlineStr">
         <is>
           <t>TIMESTAMPTZ</t>
         </is>
       </c>
-      <c r="C86" s="27" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D86" s="28" t="inlineStr">
+      <c r="C101" s="27" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D101" s="28" t="inlineStr">
         <is>
           <t>default now()</t>
         </is>
       </c>
     </row>
-    <row r="89" ht="24" customHeight="1">
-      <c r="A89" s="39" t="inlineStr">
+    <row r="104" ht="24" customHeight="1">
+      <c r="A104" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">  workflow_assignments</t>
         </is>
       </c>
     </row>
-    <row r="90" ht="30" customHeight="1">
-      <c r="A90" s="20" t="inlineStr">
+    <row r="105" ht="30" customHeight="1">
+      <c r="A105" s="20" t="inlineStr">
         <is>
           <t xml:space="preserve">  Maps each process/request_type to its active workflow — tells the engine which workflow to trigger</t>
         </is>
       </c>
     </row>
-    <row r="91" ht="18" customHeight="1">
-      <c r="A91" s="21" t="inlineStr">
+    <row r="106" ht="18" customHeight="1">
+      <c r="A106" s="21" t="inlineStr">
         <is>
           <t>Column</t>
         </is>
       </c>
-      <c r="B91" s="21" t="inlineStr">
+      <c r="B106" s="21" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="C91" s="21" t="inlineStr">
+      <c r="C106" s="21" t="inlineStr">
         <is>
           <t>Nullable</t>
         </is>
       </c>
-      <c r="D91" s="21" t="inlineStr">
+      <c r="D106" s="21" t="inlineStr">
         <is>
           <t>Notes / FK</t>
         </is>
       </c>
     </row>
-    <row r="92" ht="17" customHeight="1">
-      <c r="A92" s="22" t="inlineStr">
+    <row r="107" ht="17" customHeight="1">
+      <c r="A107" s="22" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B92" s="23" t="inlineStr">
+      <c r="B107" s="23" t="inlineStr">
         <is>
           <t>SERIAL</t>
         </is>
       </c>
-      <c r="C92" s="24" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D92" s="25" t="inlineStr">
+      <c r="C107" s="24" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D107" s="25" t="inlineStr">
         <is>
           <t>PK</t>
         </is>
       </c>
     </row>
-    <row r="93" ht="17" customHeight="1">
-      <c r="A93" s="26" t="inlineStr">
+    <row r="108" ht="17" customHeight="1">
+      <c r="A108" s="26" t="inlineStr">
         <is>
           <t>request_type</t>
         </is>
       </c>
-      <c r="B93" s="26" t="inlineStr">
+      <c r="B108" s="26" t="inlineStr">
         <is>
           <t>VARCHAR(50)</t>
         </is>
       </c>
-      <c r="C93" s="27" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D93" s="28" t="inlineStr">
+      <c r="C108" s="27" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D108" s="28" t="inlineStr">
         <is>
           <t>UNIQUE  procurement | asset</t>
         </is>
       </c>
     </row>
-    <row r="94" ht="17" customHeight="1">
-      <c r="A94" s="32" t="inlineStr">
+    <row r="109" ht="17" customHeight="1">
+      <c r="A109" s="32" t="inlineStr">
         <is>
           <t>workflow_id</t>
         </is>
       </c>
-      <c r="B94" s="33" t="inlineStr">
+      <c r="B109" s="33" t="inlineStr">
         <is>
           <t>INT</t>
         </is>
       </c>
-      <c r="C94" s="34" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D94" s="35" t="inlineStr">
+      <c r="C109" s="34" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D109" s="35" t="inlineStr">
         <is>
           <t>FK → approval_workflows.id</t>
         </is>
       </c>
     </row>
-    <row r="95" ht="17" customHeight="1">
-      <c r="A95" s="26" t="inlineStr">
+    <row r="110" ht="17" customHeight="1">
+      <c r="A110" s="26" t="inlineStr">
         <is>
           <t>is_active</t>
         </is>
       </c>
-      <c r="B95" s="26" t="inlineStr">
+      <c r="B110" s="26" t="inlineStr">
         <is>
           <t>BOOLEAN</t>
         </is>
       </c>
-      <c r="C95" s="27" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D95" s="28" t="inlineStr">
+      <c r="C110" s="27" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D110" s="28" t="inlineStr">
         <is>
           <t>default true</t>
         </is>
       </c>
     </row>
-    <row r="96" ht="17" customHeight="1">
-      <c r="A96" s="32" t="inlineStr">
+    <row r="111" ht="17" customHeight="1">
+      <c r="A111" s="32" t="inlineStr">
         <is>
           <t>updated_by</t>
         </is>
       </c>
-      <c r="B96" s="33" t="inlineStr">
+      <c r="B111" s="33" t="inlineStr">
         <is>
           <t>INT</t>
         </is>
       </c>
-      <c r="C96" s="34" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D96" s="35" t="inlineStr">
+      <c r="C111" s="34" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D111" s="35" t="inlineStr">
         <is>
           <t>FK → employees.id</t>
         </is>
       </c>
     </row>
-    <row r="97" ht="17" customHeight="1">
-      <c r="A97" s="26" t="inlineStr">
+    <row r="112" ht="17" customHeight="1">
+      <c r="A112" s="26" t="inlineStr">
         <is>
           <t>updated_at</t>
         </is>
       </c>
-      <c r="B97" s="26" t="inlineStr">
+      <c r="B112" s="26" t="inlineStr">
         <is>
           <t>TIMESTAMPTZ</t>
         </is>
       </c>
-      <c r="C97" s="27" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D97" s="28" t="inlineStr">
+      <c r="C112" s="27" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D112" s="28" t="inlineStr">
         <is>
           <t>default now()</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="17">
-    <mergeCell ref="A80:D80"/>
+  <mergeCells count="19">
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A96:D96"/>
+    <mergeCell ref="A68:D68"/>
+    <mergeCell ref="A13:D13"/>
+    <mergeCell ref="A31:D31"/>
+    <mergeCell ref="A83:D83"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A69:D69"/>
+    <mergeCell ref="A46:D46"/>
+    <mergeCell ref="A84:D84"/>
     <mergeCell ref="A56:D56"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A31:D31"/>
-    <mergeCell ref="A89:D89"/>
-    <mergeCell ref="A69:D69"/>
-    <mergeCell ref="A68:D68"/>
-    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A105:D105"/>
     <mergeCell ref="A3:D3"/>
-    <mergeCell ref="A90:D90"/>
+    <mergeCell ref="A104:D104"/>
     <mergeCell ref="A57:D57"/>
-    <mergeCell ref="A81:D81"/>
+    <mergeCell ref="A95:D95"/>
     <mergeCell ref="A47:D47"/>
-    <mergeCell ref="A46:D46"/>
     <mergeCell ref="A32:D32"/>
-    <mergeCell ref="A13:D13"/>
     <mergeCell ref="A14:D14"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4530,7 +4734,7 @@
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Unified registry of every request across all processes — powers the All Requests dashboard view</t>
+          <t xml:space="preserve">  Unified registry of every request across all processes — powers the All Requests dashboard. Updated on each status change.</t>
         </is>
       </c>
     </row>
@@ -4581,7 +4785,7 @@
     <row r="7" ht="17" customHeight="1">
       <c r="A7" s="26" t="inlineStr">
         <is>
-          <t>request_no</t>
+          <t>reference</t>
         </is>
       </c>
       <c r="B7" s="26" t="inlineStr">
@@ -4596,7 +4800,7 @@
       </c>
       <c r="D7" s="28" t="inlineStr">
         <is>
-          <t>UNIQUE  e.g. PR-2026-001, AR-2026-001</t>
+          <t>UNIQUE  e.g. PR-2026-001, AR-2026-001  — human-readable identifier shown to users</t>
         </is>
       </c>
     </row>
@@ -4806,7 +5010,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G80"/>
+  <dimension ref="A1:G63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -4832,7 +5036,7 @@
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Approved supplier/vendor registry</t>
+          <t xml:space="preserve">  Unified vendor registry — permanent (approved company suppliers) and temporary (ad-hoc one-time vendors entered at request time). Filter by vendor_type to separate them. procurement_request_id is null for permanent vendors.</t>
         </is>
       </c>
     </row>
@@ -4883,12 +5087,12 @@
     <row r="7" ht="17" customHeight="1">
       <c r="A7" s="26" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>vendor_type</t>
         </is>
       </c>
       <c r="B7" s="26" t="inlineStr">
         <is>
-          <t>VARCHAR(200)</t>
+          <t>VARCHAR(15)</t>
         </is>
       </c>
       <c r="C7" s="27" t="inlineStr">
@@ -4896,22 +5100,26 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="D7" s="28" t="inlineStr"/>
+      <c r="D7" s="28" t="inlineStr">
+        <is>
+          <t>permanent | temporary</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="17" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>contact_name</t>
+          <t>name</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>VARCHAR(150)</t>
-        </is>
-      </c>
-      <c r="C8" s="31" t="inlineStr">
-        <is>
-          <t>YES</t>
+          <t>VARCHAR(200)</t>
+        </is>
+      </c>
+      <c r="C8" s="29" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
       <c r="D8" s="30" t="inlineStr"/>
@@ -4919,7 +5127,7 @@
     <row r="9" ht="17" customHeight="1">
       <c r="A9" s="26" t="inlineStr">
         <is>
-          <t>email</t>
+          <t>contact_name</t>
         </is>
       </c>
       <c r="B9" s="26" t="inlineStr">
@@ -4937,12 +5145,12 @@
     <row r="10" ht="17" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>phone</t>
+          <t>email</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>VARCHAR(20)</t>
+          <t>VARCHAR(150)</t>
         </is>
       </c>
       <c r="C10" s="31" t="inlineStr">
@@ -4955,12 +5163,12 @@
     <row r="11" ht="17" customHeight="1">
       <c r="A11" s="26" t="inlineStr">
         <is>
-          <t>address</t>
+          <t>phone</t>
         </is>
       </c>
       <c r="B11" s="26" t="inlineStr">
         <is>
-          <t>TEXT</t>
+          <t>VARCHAR(20)</t>
         </is>
       </c>
       <c r="C11" s="38" t="inlineStr">
@@ -4973,12 +5181,12 @@
     <row r="12" ht="17" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>bank_name</t>
+          <t>address</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>VARCHAR(100)</t>
+          <t>TEXT</t>
         </is>
       </c>
       <c r="C12" s="31" t="inlineStr">
@@ -4991,12 +5199,12 @@
     <row r="13" ht="17" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>bank_account_no</t>
+          <t>bank_name</t>
         </is>
       </c>
       <c r="B13" s="26" t="inlineStr">
         <is>
-          <t>VARCHAR(30)</t>
+          <t>VARCHAR(100)</t>
         </is>
       </c>
       <c r="C13" s="38" t="inlineStr">
@@ -5009,12 +5217,12 @@
     <row r="14" ht="17" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>bank_account_name</t>
+          <t>bank_account_no</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>VARCHAR(150)</t>
+          <t>VARCHAR(30)</t>
         </is>
       </c>
       <c r="C14" s="31" t="inlineStr">
@@ -5027,319 +5235,331 @@
     <row r="15" ht="17" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
+          <t>bank_account_name</t>
+        </is>
+      </c>
+      <c r="B15" s="26" t="inlineStr">
+        <is>
+          <t>VARCHAR(150)</t>
+        </is>
+      </c>
+      <c r="C15" s="38" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D15" s="28" t="inlineStr"/>
+    </row>
+    <row r="16" ht="17" customHeight="1">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>reason</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="C16" s="31" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D16" s="30" t="inlineStr">
+        <is>
+          <t>why a registered vendor was not used — populated for temporary vendors only</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="17" customHeight="1">
+      <c r="A17" s="32" t="inlineStr">
+        <is>
+          <t>procurement_request_id</t>
+        </is>
+      </c>
+      <c r="B17" s="33" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="C17" s="36" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D17" s="35" t="inlineStr">
+        <is>
+          <t>FK → procurement_requests.id  (null for permanent vendors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="17" customHeight="1">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
           <t>is_active</t>
         </is>
       </c>
-      <c r="B15" s="26" t="inlineStr">
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t>BOOLEAN</t>
         </is>
       </c>
-      <c r="C15" s="27" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D15" s="28" t="inlineStr">
-        <is>
-          <t>default true</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="17" customHeight="1">
-      <c r="A16" s="32" t="inlineStr">
+      <c r="C18" s="29" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D18" s="30" t="inlineStr">
+        <is>
+          <t>default true — set false to deactivate a permanent vendor</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="17" customHeight="1">
+      <c r="A19" s="32" t="inlineStr">
         <is>
           <t>added_by</t>
         </is>
       </c>
-      <c r="B16" s="33" t="inlineStr">
+      <c r="B19" s="33" t="inlineStr">
         <is>
           <t>INT</t>
         </is>
       </c>
-      <c r="C16" s="34" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D16" s="35" t="inlineStr">
+      <c r="C19" s="34" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D19" s="35" t="inlineStr">
         <is>
           <t>FK → employees.id</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="17" customHeight="1">
-      <c r="A17" s="26" t="inlineStr">
+    <row r="20" ht="17" customHeight="1">
+      <c r="A20" s="5" t="inlineStr">
         <is>
           <t>created_at</t>
         </is>
       </c>
-      <c r="B17" s="26" t="inlineStr">
+      <c r="B20" s="5" t="inlineStr">
         <is>
           <t>TIMESTAMPTZ</t>
         </is>
       </c>
-      <c r="C17" s="27" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D17" s="28" t="inlineStr">
+      <c r="C20" s="29" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D20" s="30" t="inlineStr">
         <is>
           <t>default now()</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="24" customHeight="1">
-      <c r="A20" s="41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  one_time_vendors</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="30" customHeight="1">
-      <c r="A21" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Temporary/ad-hoc vendors entered at request time — not part of the approved vendor registry</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="21" t="inlineStr">
+    <row r="23" ht="24" customHeight="1">
+      <c r="A23" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  procurement_requests</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="30" customHeight="1">
+      <c r="A24" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Purchase/procurement request raised by any employee</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="21" t="inlineStr">
         <is>
           <t>Column</t>
         </is>
       </c>
-      <c r="B22" s="21" t="inlineStr">
+      <c r="B25" s="21" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="C22" s="21" t="inlineStr">
+      <c r="C25" s="21" t="inlineStr">
         <is>
           <t>Nullable</t>
         </is>
       </c>
-      <c r="D22" s="21" t="inlineStr">
+      <c r="D25" s="21" t="inlineStr">
         <is>
           <t>Notes / FK</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="17" customHeight="1">
-      <c r="A23" s="22" t="inlineStr">
+    <row r="26" ht="17" customHeight="1">
+      <c r="A26" s="22" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B23" s="23" t="inlineStr">
+      <c r="B26" s="23" t="inlineStr">
         <is>
           <t>SERIAL</t>
         </is>
       </c>
-      <c r="C23" s="24" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D23" s="25" t="inlineStr">
+      <c r="C26" s="24" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D26" s="25" t="inlineStr">
         <is>
           <t>PK</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="17" customHeight="1">
-      <c r="A24" s="32" t="inlineStr">
-        <is>
-          <t>procurement_request_id</t>
-        </is>
-      </c>
-      <c r="B24" s="33" t="inlineStr">
+    <row r="27" ht="17" customHeight="1">
+      <c r="A27" s="26" t="inlineStr">
+        <is>
+          <t>reference</t>
+        </is>
+      </c>
+      <c r="B27" s="26" t="inlineStr">
+        <is>
+          <t>VARCHAR(20)</t>
+        </is>
+      </c>
+      <c r="C27" s="27" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D27" s="28" t="inlineStr">
+        <is>
+          <t>UNIQUE  e.g. PR-2026-001  — human-readable identifier shown to users</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="17" customHeight="1">
+      <c r="A28" s="32" t="inlineStr">
+        <is>
+          <t>raised_by</t>
+        </is>
+      </c>
+      <c r="B28" s="33" t="inlineStr">
         <is>
           <t>INT</t>
         </is>
       </c>
-      <c r="C24" s="34" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D24" s="35" t="inlineStr">
-        <is>
-          <t>FK → procurement_requests.id</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="17" customHeight="1">
-      <c r="A25" s="5" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="B25" s="5" t="inlineStr">
+      <c r="C28" s="34" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D28" s="35" t="inlineStr">
+        <is>
+          <t>FK → employees.id</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="17" customHeight="1">
+      <c r="A29" s="26" t="inlineStr">
+        <is>
+          <t>department</t>
+        </is>
+      </c>
+      <c r="B29" s="26" t="inlineStr">
+        <is>
+          <t>VARCHAR(100)</t>
+        </is>
+      </c>
+      <c r="C29" s="27" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D29" s="28" t="inlineStr"/>
+    </row>
+    <row r="30" ht="17" customHeight="1">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
         <is>
           <t>VARCHAR(200)</t>
         </is>
       </c>
-      <c r="C25" s="29" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D25" s="30" t="inlineStr"/>
-    </row>
-    <row r="26" ht="17" customHeight="1">
-      <c r="A26" s="26" t="inlineStr">
-        <is>
-          <t>contact_name</t>
-        </is>
-      </c>
-      <c r="B26" s="26" t="inlineStr">
-        <is>
-          <t>VARCHAR(150)</t>
-        </is>
-      </c>
-      <c r="C26" s="38" t="inlineStr">
+      <c r="C30" s="29" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D30" s="30" t="inlineStr"/>
+    </row>
+    <row r="31" ht="17" customHeight="1">
+      <c r="A31" s="26" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="B31" s="26" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="C31" s="38" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="D26" s="28" t="inlineStr"/>
-    </row>
-    <row r="27" ht="17" customHeight="1">
-      <c r="A27" s="5" t="inlineStr">
-        <is>
-          <t>email</t>
-        </is>
-      </c>
-      <c r="B27" s="5" t="inlineStr">
-        <is>
-          <t>VARCHAR(150)</t>
-        </is>
-      </c>
-      <c r="C27" s="31" t="inlineStr">
+      <c r="D31" s="28" t="inlineStr"/>
+    </row>
+    <row r="32" ht="17" customHeight="1">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>estimated_amount</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>NUMERIC(15,2)</t>
+        </is>
+      </c>
+      <c r="C32" s="31" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="D27" s="30" t="inlineStr"/>
-    </row>
-    <row r="28" ht="17" customHeight="1">
-      <c r="A28" s="26" t="inlineStr">
-        <is>
-          <t>phone</t>
-        </is>
-      </c>
-      <c r="B28" s="26" t="inlineStr">
-        <is>
-          <t>VARCHAR(20)</t>
-        </is>
-      </c>
-      <c r="C28" s="38" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="D28" s="28" t="inlineStr"/>
-    </row>
-    <row r="29" ht="17" customHeight="1">
-      <c r="A29" s="5" t="inlineStr">
-        <is>
-          <t>address</t>
-        </is>
-      </c>
-      <c r="B29" s="5" t="inlineStr">
-        <is>
-          <t>TEXT</t>
-        </is>
-      </c>
-      <c r="C29" s="31" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="D29" s="30" t="inlineStr"/>
-    </row>
-    <row r="30" ht="17" customHeight="1">
-      <c r="A30" s="26" t="inlineStr">
-        <is>
-          <t>bank_name</t>
-        </is>
-      </c>
-      <c r="B30" s="26" t="inlineStr">
-        <is>
-          <t>VARCHAR(100)</t>
-        </is>
-      </c>
-      <c r="C30" s="38" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="D30" s="28" t="inlineStr"/>
-    </row>
-    <row r="31" ht="17" customHeight="1">
-      <c r="A31" s="5" t="inlineStr">
-        <is>
-          <t>bank_account_no</t>
-        </is>
-      </c>
-      <c r="B31" s="5" t="inlineStr">
-        <is>
-          <t>VARCHAR(30)</t>
-        </is>
-      </c>
-      <c r="C31" s="31" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="D31" s="30" t="inlineStr"/>
-    </row>
-    <row r="32" ht="17" customHeight="1">
-      <c r="A32" s="26" t="inlineStr">
-        <is>
-          <t>bank_account_name</t>
-        </is>
-      </c>
-      <c r="B32" s="26" t="inlineStr">
-        <is>
-          <t>VARCHAR(150)</t>
-        </is>
-      </c>
-      <c r="C32" s="38" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="D32" s="28" t="inlineStr"/>
+      <c r="D32" s="30" t="inlineStr"/>
     </row>
     <row r="33" ht="17" customHeight="1">
-      <c r="A33" s="5" t="inlineStr">
-        <is>
-          <t>reason</t>
-        </is>
-      </c>
-      <c r="B33" s="5" t="inlineStr">
-        <is>
-          <t>TEXT</t>
-        </is>
-      </c>
-      <c r="C33" s="31" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="D33" s="30" t="inlineStr">
-        <is>
-          <t>why a registered vendor was not used</t>
+      <c r="A33" s="26" t="inlineStr">
+        <is>
+          <t>currency</t>
+        </is>
+      </c>
+      <c r="B33" s="26" t="inlineStr">
+        <is>
+          <t>VARCHAR(5)</t>
+        </is>
+      </c>
+      <c r="C33" s="27" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D33" s="28" t="inlineStr">
+        <is>
+          <t>default NGN</t>
         </is>
       </c>
     </row>
     <row r="34" ht="17" customHeight="1">
       <c r="A34" s="32" t="inlineStr">
         <is>
-          <t>added_by</t>
+          <t>vendor_id</t>
         </is>
       </c>
       <c r="B34" s="33" t="inlineStr">
@@ -5347,168 +5567,172 @@
           <t>INT</t>
         </is>
       </c>
-      <c r="C34" s="34" t="inlineStr">
-        <is>
-          <t>NO</t>
+      <c r="C34" s="36" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
       <c r="D34" s="35" t="inlineStr">
         <is>
-          <t>FK → employees.id</t>
+          <t>FK → vendors.id  (permanent or temporary — set after vendor selection)</t>
         </is>
       </c>
     </row>
     <row r="35" ht="17" customHeight="1">
-      <c r="A35" s="5" t="inlineStr">
+      <c r="A35" s="26" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="B35" s="26" t="inlineStr">
+        <is>
+          <t>VARCHAR(20)</t>
+        </is>
+      </c>
+      <c r="C35" s="27" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D35" s="28" t="inlineStr">
+        <is>
+          <t>draft | pending | approved | rejected | returned | po_issued</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="17" customHeight="1">
+      <c r="A36" s="5" t="inlineStr">
         <is>
           <t>created_at</t>
         </is>
       </c>
-      <c r="B35" s="5" t="inlineStr">
+      <c r="B36" s="5" t="inlineStr">
         <is>
           <t>TIMESTAMPTZ</t>
         </is>
       </c>
-      <c r="C35" s="29" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D35" s="30" t="inlineStr">
+      <c r="C36" s="29" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D36" s="30" t="inlineStr">
         <is>
           <t>default now()</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="24" customHeight="1">
-      <c r="A38" s="41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  procurement_requests</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="30" customHeight="1">
-      <c r="A39" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Purchase/procurement request raised by any employee</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="18" customHeight="1">
-      <c r="A40" s="21" t="inlineStr">
+    <row r="37" ht="17" customHeight="1">
+      <c r="A37" s="26" t="inlineStr">
+        <is>
+          <t>updated_at</t>
+        </is>
+      </c>
+      <c r="B37" s="26" t="inlineStr">
+        <is>
+          <t>TIMESTAMPTZ</t>
+        </is>
+      </c>
+      <c r="C37" s="27" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D37" s="28" t="inlineStr">
+        <is>
+          <t>default now()</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="24" customHeight="1">
+      <c r="A40" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  procurement_items</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="30" customHeight="1">
+      <c r="A41" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Line items on a procurement request</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="18" customHeight="1">
+      <c r="A42" s="21" t="inlineStr">
         <is>
           <t>Column</t>
         </is>
       </c>
-      <c r="B40" s="21" t="inlineStr">
+      <c r="B42" s="21" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="C40" s="21" t="inlineStr">
+      <c r="C42" s="21" t="inlineStr">
         <is>
           <t>Nullable</t>
         </is>
       </c>
-      <c r="D40" s="21" t="inlineStr">
+      <c r="D42" s="21" t="inlineStr">
         <is>
           <t>Notes / FK</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="17" customHeight="1">
-      <c r="A41" s="22" t="inlineStr">
+    <row r="43" ht="17" customHeight="1">
+      <c r="A43" s="22" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B41" s="23" t="inlineStr">
+      <c r="B43" s="23" t="inlineStr">
         <is>
           <t>SERIAL</t>
         </is>
       </c>
-      <c r="C41" s="24" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D41" s="25" t="inlineStr">
+      <c r="C43" s="24" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D43" s="25" t="inlineStr">
         <is>
           <t>PK</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="17" customHeight="1">
-      <c r="A42" s="26" t="inlineStr">
-        <is>
-          <t>request_no</t>
-        </is>
-      </c>
-      <c r="B42" s="26" t="inlineStr">
-        <is>
-          <t>VARCHAR(20)</t>
-        </is>
-      </c>
-      <c r="C42" s="27" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D42" s="28" t="inlineStr">
-        <is>
-          <t>UNIQUE  e.g. PR-2026-001</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="17" customHeight="1">
-      <c r="A43" s="32" t="inlineStr">
-        <is>
-          <t>raised_by</t>
-        </is>
-      </c>
-      <c r="B43" s="33" t="inlineStr">
+    <row r="44" ht="17" customHeight="1">
+      <c r="A44" s="32" t="inlineStr">
+        <is>
+          <t>procurement_request_id</t>
+        </is>
+      </c>
+      <c r="B44" s="33" t="inlineStr">
         <is>
           <t>INT</t>
         </is>
       </c>
-      <c r="C43" s="34" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D43" s="35" t="inlineStr">
-        <is>
-          <t>FK → employees.id</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="17" customHeight="1">
-      <c r="A44" s="26" t="inlineStr">
-        <is>
-          <t>department</t>
-        </is>
-      </c>
-      <c r="B44" s="26" t="inlineStr">
-        <is>
-          <t>VARCHAR(100)</t>
-        </is>
-      </c>
-      <c r="C44" s="27" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D44" s="28" t="inlineStr"/>
+      <c r="C44" s="34" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D44" s="35" t="inlineStr">
+        <is>
+          <t>FK → procurement_requests.id</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="17" customHeight="1">
       <c r="A45" s="5" t="inlineStr">
         <is>
-          <t>title</t>
+          <t>description</t>
         </is>
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>VARCHAR(200)</t>
+          <t>VARCHAR(255)</t>
         </is>
       </c>
       <c r="C45" s="29" t="inlineStr">
@@ -5521,17 +5745,17 @@
     <row r="46" ht="17" customHeight="1">
       <c r="A46" s="26" t="inlineStr">
         <is>
-          <t>description</t>
+          <t>quantity</t>
         </is>
       </c>
       <c r="B46" s="26" t="inlineStr">
         <is>
-          <t>TEXT</t>
-        </is>
-      </c>
-      <c r="C46" s="38" t="inlineStr">
-        <is>
-          <t>YES</t>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="C46" s="27" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
       <c r="D46" s="28" t="inlineStr"/>
@@ -5539,7 +5763,7 @@
     <row r="47" ht="17" customHeight="1">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>estimated_amount</t>
+          <t>unit_price</t>
         </is>
       </c>
       <c r="B47" s="5" t="inlineStr">
@@ -5557,197 +5781,193 @@
     <row r="48" ht="17" customHeight="1">
       <c r="A48" s="26" t="inlineStr">
         <is>
+          <t>total_price</t>
+        </is>
+      </c>
+      <c r="B48" s="26" t="inlineStr">
+        <is>
+          <t>NUMERIC(15,2)</t>
+        </is>
+      </c>
+      <c r="C48" s="38" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D48" s="28" t="inlineStr">
+        <is>
+          <t>computed: qty × unit_price</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="24" customHeight="1">
+      <c r="A51" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  purchase_orders</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="30" customHeight="1">
+      <c r="A52" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  PO issued after procurement request is fully approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="18" customHeight="1">
+      <c r="A53" s="21" t="inlineStr">
+        <is>
+          <t>Column</t>
+        </is>
+      </c>
+      <c r="B53" s="21" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C53" s="21" t="inlineStr">
+        <is>
+          <t>Nullable</t>
+        </is>
+      </c>
+      <c r="D53" s="21" t="inlineStr">
+        <is>
+          <t>Notes / FK</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="17" customHeight="1">
+      <c r="A54" s="22" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B54" s="23" t="inlineStr">
+        <is>
+          <t>SERIAL</t>
+        </is>
+      </c>
+      <c r="C54" s="24" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D54" s="25" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="17" customHeight="1">
+      <c r="A55" s="26" t="inlineStr">
+        <is>
+          <t>po_number</t>
+        </is>
+      </c>
+      <c r="B55" s="26" t="inlineStr">
+        <is>
+          <t>VARCHAR(20)</t>
+        </is>
+      </c>
+      <c r="C55" s="27" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D55" s="28" t="inlineStr">
+        <is>
+          <t>UNIQUE  e.g. PO-2026-001</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="17" customHeight="1">
+      <c r="A56" s="32" t="inlineStr">
+        <is>
+          <t>procurement_request_id</t>
+        </is>
+      </c>
+      <c r="B56" s="33" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="C56" s="34" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D56" s="35" t="inlineStr">
+        <is>
+          <t>FK → procurement_requests.id</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="17" customHeight="1">
+      <c r="A57" s="32" t="inlineStr">
+        <is>
+          <t>vendor_id</t>
+        </is>
+      </c>
+      <c r="B57" s="33" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="C57" s="34" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D57" s="35" t="inlineStr">
+        <is>
+          <t>FK → vendors.id  (permanent or temporary)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="17" customHeight="1">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>total_amount</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="inlineStr">
+        <is>
+          <t>NUMERIC(15,2)</t>
+        </is>
+      </c>
+      <c r="C58" s="29" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D58" s="30" t="inlineStr"/>
+    </row>
+    <row r="59" ht="17" customHeight="1">
+      <c r="A59" s="26" t="inlineStr">
+        <is>
           <t>currency</t>
         </is>
       </c>
-      <c r="B48" s="26" t="inlineStr">
+      <c r="B59" s="26" t="inlineStr">
         <is>
           <t>VARCHAR(5)</t>
         </is>
       </c>
-      <c r="C48" s="27" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D48" s="28" t="inlineStr">
+      <c r="C59" s="27" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D59" s="28" t="inlineStr">
         <is>
           <t>default NGN</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="17" customHeight="1">
-      <c r="A49" s="5" t="inlineStr">
-        <is>
-          <t>vendor_type</t>
-        </is>
-      </c>
-      <c r="B49" s="5" t="inlineStr">
-        <is>
-          <t>VARCHAR(20)</t>
-        </is>
-      </c>
-      <c r="C49" s="31" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="D49" s="30" t="inlineStr">
-        <is>
-          <t>registered | one_time</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="17" customHeight="1">
-      <c r="A50" s="32" t="inlineStr">
-        <is>
-          <t>vendor_id</t>
-        </is>
-      </c>
-      <c r="B50" s="33" t="inlineStr">
-        <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="C50" s="36" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="D50" s="35" t="inlineStr">
-        <is>
-          <t>FK → vendors.id  (null if one_time)</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="17" customHeight="1">
-      <c r="A51" s="5" t="inlineStr">
-        <is>
-          <t>status</t>
-        </is>
-      </c>
-      <c r="B51" s="5" t="inlineStr">
-        <is>
-          <t>VARCHAR(20)</t>
-        </is>
-      </c>
-      <c r="C51" s="29" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D51" s="30" t="inlineStr">
-        <is>
-          <t>draft | pending | approved | rejected | returned | po_issued</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="17" customHeight="1">
-      <c r="A52" s="26" t="inlineStr">
-        <is>
-          <t>created_at</t>
-        </is>
-      </c>
-      <c r="B52" s="26" t="inlineStr">
-        <is>
-          <t>TIMESTAMPTZ</t>
-        </is>
-      </c>
-      <c r="C52" s="27" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D52" s="28" t="inlineStr">
-        <is>
-          <t>default now()</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="17" customHeight="1">
-      <c r="A53" s="5" t="inlineStr">
-        <is>
-          <t>updated_at</t>
-        </is>
-      </c>
-      <c r="B53" s="5" t="inlineStr">
-        <is>
-          <t>TIMESTAMPTZ</t>
-        </is>
-      </c>
-      <c r="C53" s="29" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D53" s="30" t="inlineStr">
-        <is>
-          <t>default now()</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" ht="24" customHeight="1">
-      <c r="A56" s="41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  procurement_items</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" ht="30" customHeight="1">
-      <c r="A57" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Line items on a procurement request</t>
-        </is>
-      </c>
-    </row>
-    <row r="58" ht="18" customHeight="1">
-      <c r="A58" s="21" t="inlineStr">
-        <is>
-          <t>Column</t>
-        </is>
-      </c>
-      <c r="B58" s="21" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="C58" s="21" t="inlineStr">
-        <is>
-          <t>Nullable</t>
-        </is>
-      </c>
-      <c r="D58" s="21" t="inlineStr">
-        <is>
-          <t>Notes / FK</t>
-        </is>
-      </c>
-    </row>
-    <row r="59" ht="17" customHeight="1">
-      <c r="A59" s="22" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="B59" s="23" t="inlineStr">
-        <is>
-          <t>SERIAL</t>
-        </is>
-      </c>
-      <c r="C59" s="24" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D59" s="25" t="inlineStr">
-        <is>
-          <t>PK</t>
         </is>
       </c>
     </row>
     <row r="60" ht="17" customHeight="1">
       <c r="A60" s="32" t="inlineStr">
         <is>
-          <t>procurement_request_id</t>
+          <t>issued_by</t>
         </is>
       </c>
       <c r="B60" s="33" t="inlineStr">
@@ -5762,369 +5982,83 @@
       </c>
       <c r="D60" s="35" t="inlineStr">
         <is>
-          <t>FK → procurement_requests.id</t>
+          <t>FK → employees.id</t>
         </is>
       </c>
     </row>
     <row r="61" ht="17" customHeight="1">
-      <c r="A61" s="5" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="B61" s="5" t="inlineStr">
-        <is>
-          <t>VARCHAR(255)</t>
-        </is>
-      </c>
-      <c r="C61" s="29" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D61" s="30" t="inlineStr"/>
+      <c r="A61" s="26" t="inlineStr">
+        <is>
+          <t>issued_at</t>
+        </is>
+      </c>
+      <c r="B61" s="26" t="inlineStr">
+        <is>
+          <t>TIMESTAMPTZ</t>
+        </is>
+      </c>
+      <c r="C61" s="27" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D61" s="28" t="inlineStr">
+        <is>
+          <t>default now()</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="17" customHeight="1">
-      <c r="A62" s="26" t="inlineStr">
-        <is>
-          <t>quantity</t>
-        </is>
-      </c>
-      <c r="B62" s="26" t="inlineStr">
-        <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="C62" s="27" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D62" s="28" t="inlineStr"/>
+      <c r="A62" s="5" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="B62" s="5" t="inlineStr">
+        <is>
+          <t>VARCHAR(20)</t>
+        </is>
+      </c>
+      <c r="C62" s="29" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D62" s="30" t="inlineStr">
+        <is>
+          <t>issued | delivered | cancelled</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="17" customHeight="1">
-      <c r="A63" s="5" t="inlineStr">
-        <is>
-          <t>unit_price</t>
-        </is>
-      </c>
-      <c r="B63" s="5" t="inlineStr">
-        <is>
-          <t>NUMERIC(15,2)</t>
-        </is>
-      </c>
-      <c r="C63" s="31" t="inlineStr">
+      <c r="A63" s="26" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+      <c r="B63" s="26" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="C63" s="38" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="D63" s="30" t="inlineStr"/>
-    </row>
-    <row r="64" ht="17" customHeight="1">
-      <c r="A64" s="26" t="inlineStr">
-        <is>
-          <t>total_price</t>
-        </is>
-      </c>
-      <c r="B64" s="26" t="inlineStr">
-        <is>
-          <t>NUMERIC(15,2)</t>
-        </is>
-      </c>
-      <c r="C64" s="38" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="D64" s="28" t="inlineStr">
-        <is>
-          <t>computed: qty × unit_price</t>
-        </is>
-      </c>
-    </row>
-    <row r="67" ht="24" customHeight="1">
-      <c r="A67" s="41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  purchase_orders</t>
-        </is>
-      </c>
-    </row>
-    <row r="68" ht="30" customHeight="1">
-      <c r="A68" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  PO issued after procurement request is fully approved</t>
-        </is>
-      </c>
-    </row>
-    <row r="69" ht="18" customHeight="1">
-      <c r="A69" s="21" t="inlineStr">
-        <is>
-          <t>Column</t>
-        </is>
-      </c>
-      <c r="B69" s="21" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="C69" s="21" t="inlineStr">
-        <is>
-          <t>Nullable</t>
-        </is>
-      </c>
-      <c r="D69" s="21" t="inlineStr">
-        <is>
-          <t>Notes / FK</t>
-        </is>
-      </c>
-    </row>
-    <row r="70" ht="17" customHeight="1">
-      <c r="A70" s="22" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="B70" s="23" t="inlineStr">
-        <is>
-          <t>SERIAL</t>
-        </is>
-      </c>
-      <c r="C70" s="24" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D70" s="25" t="inlineStr">
-        <is>
-          <t>PK</t>
-        </is>
-      </c>
-    </row>
-    <row r="71" ht="17" customHeight="1">
-      <c r="A71" s="26" t="inlineStr">
-        <is>
-          <t>po_number</t>
-        </is>
-      </c>
-      <c r="B71" s="26" t="inlineStr">
-        <is>
-          <t>VARCHAR(20)</t>
-        </is>
-      </c>
-      <c r="C71" s="27" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D71" s="28" t="inlineStr">
-        <is>
-          <t>UNIQUE  e.g. PO-2026-001</t>
-        </is>
-      </c>
-    </row>
-    <row r="72" ht="17" customHeight="1">
-      <c r="A72" s="32" t="inlineStr">
-        <is>
-          <t>procurement_request_id</t>
-        </is>
-      </c>
-      <c r="B72" s="33" t="inlineStr">
-        <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="C72" s="34" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D72" s="35" t="inlineStr">
-        <is>
-          <t>FK → procurement_requests.id</t>
-        </is>
-      </c>
-    </row>
-    <row r="73" ht="17" customHeight="1">
-      <c r="A73" s="32" t="inlineStr">
-        <is>
-          <t>vendor_id</t>
-        </is>
-      </c>
-      <c r="B73" s="33" t="inlineStr">
-        <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="C73" s="36" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="D73" s="35" t="inlineStr">
-        <is>
-          <t>FK → vendors.id  (null if one_time_vendor used)</t>
-        </is>
-      </c>
-    </row>
-    <row r="74" ht="17" customHeight="1">
-      <c r="A74" s="32" t="inlineStr">
-        <is>
-          <t>one_time_vendor_id</t>
-        </is>
-      </c>
-      <c r="B74" s="33" t="inlineStr">
-        <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="C74" s="36" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="D74" s="35" t="inlineStr">
-        <is>
-          <t>FK → one_time_vendors.id  (null if registered vendor used)</t>
-        </is>
-      </c>
-    </row>
-    <row r="75" ht="17" customHeight="1">
-      <c r="A75" s="26" t="inlineStr">
-        <is>
-          <t>total_amount</t>
-        </is>
-      </c>
-      <c r="B75" s="26" t="inlineStr">
-        <is>
-          <t>NUMERIC(15,2)</t>
-        </is>
-      </c>
-      <c r="C75" s="27" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D75" s="28" t="inlineStr"/>
-    </row>
-    <row r="76" ht="17" customHeight="1">
-      <c r="A76" s="5" t="inlineStr">
-        <is>
-          <t>currency</t>
-        </is>
-      </c>
-      <c r="B76" s="5" t="inlineStr">
-        <is>
-          <t>VARCHAR(5)</t>
-        </is>
-      </c>
-      <c r="C76" s="29" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D76" s="30" t="inlineStr">
-        <is>
-          <t>default NGN</t>
-        </is>
-      </c>
-    </row>
-    <row r="77" ht="17" customHeight="1">
-      <c r="A77" s="32" t="inlineStr">
-        <is>
-          <t>issued_by</t>
-        </is>
-      </c>
-      <c r="B77" s="33" t="inlineStr">
-        <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="C77" s="34" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D77" s="35" t="inlineStr">
-        <is>
-          <t>FK → employees.id</t>
-        </is>
-      </c>
-    </row>
-    <row r="78" ht="17" customHeight="1">
-      <c r="A78" s="5" t="inlineStr">
-        <is>
-          <t>issued_at</t>
-        </is>
-      </c>
-      <c r="B78" s="5" t="inlineStr">
-        <is>
-          <t>TIMESTAMPTZ</t>
-        </is>
-      </c>
-      <c r="C78" s="29" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D78" s="30" t="inlineStr">
-        <is>
-          <t>default now()</t>
-        </is>
-      </c>
-    </row>
-    <row r="79" ht="17" customHeight="1">
-      <c r="A79" s="26" t="inlineStr">
-        <is>
-          <t>status</t>
-        </is>
-      </c>
-      <c r="B79" s="26" t="inlineStr">
-        <is>
-          <t>VARCHAR(20)</t>
-        </is>
-      </c>
-      <c r="C79" s="27" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D79" s="28" t="inlineStr">
-        <is>
-          <t>issued | delivered | cancelled</t>
-        </is>
-      </c>
-    </row>
-    <row r="80" ht="17" customHeight="1">
-      <c r="A80" s="5" t="inlineStr">
-        <is>
-          <t>notes</t>
-        </is>
-      </c>
-      <c r="B80" s="5" t="inlineStr">
-        <is>
-          <t>TEXT</t>
-        </is>
-      </c>
-      <c r="C80" s="31" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="D80" s="30" t="inlineStr"/>
+      <c r="D63" s="28" t="inlineStr"/>
     </row>
   </sheetData>
-  <mergeCells count="11">
-    <mergeCell ref="A56:D56"/>
-    <mergeCell ref="A67:D67"/>
+  <mergeCells count="9">
+    <mergeCell ref="A23:D23"/>
+    <mergeCell ref="A40:D40"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A4:D4"/>
     <mergeCell ref="A3:D3"/>
-    <mergeCell ref="A20:D20"/>
-    <mergeCell ref="A21:D21"/>
-    <mergeCell ref="A38:D38"/>
-    <mergeCell ref="A39:D39"/>
-    <mergeCell ref="A57:D57"/>
-    <mergeCell ref="A68:D68"/>
+    <mergeCell ref="A52:D52"/>
+    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="A41:D41"/>
+    <mergeCell ref="A51:D51"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6667,7 +6601,7 @@
     <row r="36" ht="17" customHeight="1">
       <c r="A36" s="26" t="inlineStr">
         <is>
-          <t>request_no</t>
+          <t>reference</t>
         </is>
       </c>
       <c r="B36" s="26" t="inlineStr">
@@ -6682,7 +6616,7 @@
       </c>
       <c r="D36" s="28" t="inlineStr">
         <is>
-          <t>UNIQUE  e.g. AR-2026-001</t>
+          <t>UNIQUE  e.g. AR-2026-001  — human-readable identifier shown to users</t>
         </is>
       </c>
     </row>

</xml_diff>